<commit_message>
Rename two lookalike Nepo cards and fix Exile's card name
Hand Me Down becomes Last Season and Hush Fund becomes Burn the Receipts, so
they no longer read as Hand-Me-Downs and Hush Money. Assets, spec, enum
comment and the art-prompt workbook follow. Exile's _cardName said "Self Pity",
so two status cards shared that name in game.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Ua161fkUnj3L57WohDdyM
</commit_message>
<xml_diff>
--- a/docs/crookedile-card-art-prompts.xlsx
+++ b/docs/crookedile-card-art-prompts.xlsx
@@ -3247,7 +3247,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Hand Me Down</t>
+          <t>Last Season</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>one oversized hand-me-down jacket flung forward with motion arcs, one emerald green accent</t>
+          <t>one last-season designer handbag flung forward with motion arcs, one emerald green accent</t>
         </is>
       </c>
       <c r="F5" s="4">
@@ -3929,7 +3929,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Hush Fund</t>
+          <t>Burn the Receipts</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>one locked safe forming a protective ring, one emerald green accent</t>
+          <t>one stack of receipts burning inside a protective ring, one emerald green accent</t>
         </is>
       </c>
       <c r="F27" s="4">

</xml_diff>

<commit_message>
Celebrity debt, glamour, and tactics
Adds the Celebrity Glamour/IOU card suite, the debt/promise rules, and new battle effects for Glamour ticks, borrowing, token replacement, and Poisoned Perception payoff. This also updates the card database, UI affordances, and docs to match the current built rules, with Play Mode tests covering the new behavior and edge cases.
</commit_message>
<xml_diff>
--- a/docs/crookedile-card-art-prompts.xlsx
+++ b/docs/crookedile-card-art-prompts.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Art Rules" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Faith Leader" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Celebrity" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Nepo Baby" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Art Rules" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faith Leader" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Celebrity" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nepo Baby" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Faith Leader'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Celebrity'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Celebrity'!$A$1:$F$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Nepo Baby'!$A$1:$F$43</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -2279,7 +2279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Rhetoric</t>
+          <t>Pressure</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Policy</t>
+          <t>Rhetoric</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -3096,8 +3096,307 @@
         <v/>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Advance Booking</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Enhanced</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Rhetoric</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E27&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Charm Offensive</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr"/>
+      <c r="F28" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E28&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Disarming Charm</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Enhanced</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Rhetoric</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr"/>
+      <c r="F29" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E29&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Iconic Line</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Enhanced</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Rhetoric</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr"/>
+      <c r="E30" s="4" t="inlineStr"/>
+      <c r="F30" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E30&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Media Training</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Enhanced</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Policy</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E31&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Movie Quote</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Token</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Rhetoric</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr"/>
+      <c r="E32" s="4" t="inlineStr"/>
+      <c r="F32" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E32&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Never Meet Your Heroes</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Enhanced</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Rhetoric</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr"/>
+      <c r="F33" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E33&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Overpromise</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Rhetoric</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr"/>
+      <c r="E34" s="4" t="inlineStr"/>
+      <c r="F34" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E34&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Paid-Off Promises</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Enhanced</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Rhetoric</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E35&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Payment Holiday</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Enhanced</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Rhetoric</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E36&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Second Take</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Enhanced</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Rhetoric</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E37&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Signature Catchphrase</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Policy</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E38&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Victim Narrative</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Enhanced</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Rhetoric</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="4">
+        <f>Settings!$B$2&amp;" - "&amp;E39&amp;", "&amp;Settings!$B$5&amp;" "&amp;Settings!$B$3&amp;IF(Settings!$B$4&lt;&gt;""," --sref "&amp;Settings!$B$4,"")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:F39"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>

</xml_diff>